<commit_message>
Steps marked with the logo's three rays; Cal.com → Google Sheets webhook script, setup guide and booking-ID column
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ttx2kJrAs6ugivvU5h1u4L
</commit_message>
<xml_diff>
--- a/docs/agencias/300sun-comisiones-agencias.xlsx
+++ b/docs/agencias/300sun-comisiones-agencias.xlsx
@@ -184,6 +184,11 @@
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
         <t>Lo que pagó el cliente por el paseo o la paella (señal + resto). Sin propinas, entradas ni comida.</t>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="0" shapeId="0">
+      <text>
+        <t>Lo rellena solo Google Sheets cuando entra una reserva desde Cal.com. No lo toques.</t>
       </text>
     </comment>
   </commentList>
@@ -499,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N301"/>
+  <dimension ref="A1:O301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -516,6 +521,7 @@
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="40" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -587,6 +593,11 @@
       <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Notas</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>ID reserva Cal.com</t>
         </is>
       </c>
     </row>

</xml_diff>